<commit_message>
Fix printer and add menu import from excel
</commit_message>
<xml_diff>
--- a/data/palacio_royal_09_12_2026.xlsx
+++ b/data/palacio_royal_09_12_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\renha\workspace\projects\big_boss_bro\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641DCCCA-D47E-4BE5-B19C-349DD65AE48E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20DFF318-170E-4CE0-94C2-DAC8772A0FDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="126">
   <si>
     <t>种类</t>
   </si>
@@ -91,16 +91,334 @@
   </si>
   <si>
     <t>Mediano/Grande</t>
+  </si>
+  <si>
+    <t>Arroz con puerco</t>
+  </si>
+  <si>
+    <t>Arroz blanco</t>
+  </si>
+  <si>
+    <t>Arroz con chorizo</t>
+  </si>
+  <si>
+    <t>Chow Mein</t>
+  </si>
+  <si>
+    <t>Chow mein cantones</t>
+  </si>
+  <si>
+    <t>Chow mein con pollo</t>
+  </si>
+  <si>
+    <t>Chow mein con res</t>
+  </si>
+  <si>
+    <t>Chow mein con camaron</t>
+  </si>
+  <si>
+    <t>He fen con res</t>
+  </si>
+  <si>
+    <t>He fen con camaron</t>
+  </si>
+  <si>
+    <t>He fen con pollo</t>
+  </si>
+  <si>
+    <t>He fen cantones</t>
+  </si>
+  <si>
+    <t>定制1选项价格</t>
+  </si>
+  <si>
+    <t>140/200</t>
+  </si>
+  <si>
+    <t>140/203</t>
+  </si>
+  <si>
+    <t>130/180</t>
+  </si>
+  <si>
+    <t>140/150</t>
+  </si>
+  <si>
+    <t>基础价格</t>
+  </si>
+  <si>
+    <t>185/240</t>
+  </si>
+  <si>
+    <t>160/220</t>
+  </si>
+  <si>
+    <t>180/240</t>
+  </si>
+  <si>
+    <t>140/185</t>
+  </si>
+  <si>
+    <t>175/250</t>
+  </si>
+  <si>
+    <t>150/200</t>
+  </si>
+  <si>
+    <t>Sizzling Hot Pot</t>
+  </si>
+  <si>
+    <t>Mariscos hot pot</t>
+  </si>
+  <si>
+    <t>Especial hot pot</t>
+  </si>
+  <si>
+    <t>Sizzling de camaron</t>
+  </si>
+  <si>
+    <t>Sizzling de pollo</t>
+  </si>
+  <si>
+    <t>Sizzling de res</t>
+  </si>
+  <si>
+    <t>Mariscos</t>
+  </si>
+  <si>
+    <t>Camaron con naranja</t>
+  </si>
+  <si>
+    <t>Camaron almendrado</t>
+  </si>
+  <si>
+    <t>Camaroncon brocoli</t>
+  </si>
+  <si>
+    <t>Camaron enchilado</t>
+  </si>
+  <si>
+    <t>Comninacion de masiscos</t>
+  </si>
+  <si>
+    <t>Calamar enchilado</t>
+  </si>
+  <si>
+    <t>200/310</t>
+  </si>
+  <si>
+    <t>200/300</t>
+  </si>
+  <si>
+    <t>Bebidas</t>
+  </si>
+  <si>
+    <t>Sodas</t>
+  </si>
+  <si>
+    <t>Te helado</t>
+  </si>
+  <si>
+    <t>Te caliente</t>
+  </si>
+  <si>
+    <t>Te caliente chino</t>
+  </si>
+  <si>
+    <t>Limonada</t>
+  </si>
+  <si>
+    <t>Limonada Mineral</t>
+  </si>
+  <si>
+    <t>Naranjada</t>
+  </si>
+  <si>
+    <t>Naranjada Mineral</t>
+  </si>
+  <si>
+    <t>Jugo de naranja</t>
+  </si>
+  <si>
+    <t>Café</t>
+  </si>
+  <si>
+    <t>Matcha Smoothie</t>
+  </si>
+  <si>
+    <t>Taro Smoothie</t>
+  </si>
+  <si>
+    <t>Chocolate Smoothie</t>
+  </si>
+  <si>
+    <t>Oreo Smoothie</t>
+  </si>
+  <si>
+    <t>Taro Boba</t>
+  </si>
+  <si>
+    <t>Matcha Boba</t>
+  </si>
+  <si>
+    <t>Jazmin Boba</t>
+  </si>
+  <si>
+    <t>Cerveza</t>
+  </si>
+  <si>
+    <t>Sapporo</t>
+  </si>
+  <si>
+    <t>Tsingtao</t>
+  </si>
+  <si>
+    <t>Clamato+Michelada</t>
+  </si>
+  <si>
+    <t>Paloma</t>
+  </si>
+  <si>
+    <t>JARRA</t>
+  </si>
+  <si>
+    <t>Yes/No</t>
+  </si>
+  <si>
+    <t>125/0</t>
+  </si>
+  <si>
+    <t>60/0</t>
+  </si>
+  <si>
+    <t>130/0</t>
+  </si>
+  <si>
+    <t>135/0</t>
+  </si>
+  <si>
+    <t>EXTRA BOBA</t>
+  </si>
+  <si>
+    <t>25/0</t>
+  </si>
+  <si>
+    <t>Tofu</t>
+  </si>
+  <si>
+    <t>Tofu de pollo</t>
+  </si>
+  <si>
+    <t>Tofu de res</t>
+  </si>
+  <si>
+    <t>Tofu de camaron</t>
+  </si>
+  <si>
+    <t>Tofu con verduras</t>
+  </si>
+  <si>
+    <t>Tofu kunpo</t>
+  </si>
+  <si>
+    <t>Botanas</t>
+  </si>
+  <si>
+    <t>Chun Kun</t>
+  </si>
+  <si>
+    <t>Chiles asados</t>
+  </si>
+  <si>
+    <t>Papas Fritas</t>
+  </si>
+  <si>
+    <t>Churritos</t>
+  </si>
+  <si>
+    <t>Queso wonto asado</t>
+  </si>
+  <si>
+    <t>Dumplings fritos / al vapor</t>
+  </si>
+  <si>
+    <t>Sesame balls</t>
+  </si>
+  <si>
+    <t>40/80</t>
+  </si>
+  <si>
+    <t>30/60</t>
+  </si>
+  <si>
+    <t>80/140</t>
+  </si>
+  <si>
+    <t>135/195</t>
+  </si>
+  <si>
+    <t>150/230</t>
+  </si>
+  <si>
+    <t>Caldos</t>
+  </si>
+  <si>
+    <t>Caldo wonton</t>
+  </si>
+  <si>
+    <t>Caldo de mariscos</t>
+  </si>
+  <si>
+    <t>Caldo de camaron</t>
+  </si>
+  <si>
+    <t>Caldo cantones</t>
+  </si>
+  <si>
+    <t>Caldo de alte</t>
+  </si>
+  <si>
+    <t>Clado mandarin</t>
+  </si>
+  <si>
+    <t>Caldo de pollo</t>
+  </si>
+  <si>
+    <t>Caldo de molleja</t>
+  </si>
+  <si>
+    <t>Caldo de verdura</t>
+  </si>
+  <si>
+    <t>Caldo con noodle solo per</t>
+  </si>
+  <si>
+    <t>Caldo con hefen chino solo por</t>
+  </si>
+  <si>
+    <t>165/250</t>
+  </si>
+  <si>
+    <t>155/230</t>
+  </si>
+  <si>
+    <t>120/180</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -408,16 +726,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="18.921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.921875" customWidth="1"/>
+    <col min="4" max="4" width="13.921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="13.921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -425,187 +745,1372 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>20</v>
+      <c r="C2">
+        <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
-        <v>20</v>
+      <c r="C3">
+        <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
-        <v>20</v>
+      <c r="C4">
+        <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" t="s">
-        <v>20</v>
+      <c r="C5">
+        <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" t="s">
-        <v>20</v>
+      <c r="C6">
+        <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" t="s">
-        <v>20</v>
+      <c r="C7">
+        <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="E7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" t="s">
-        <v>20</v>
+      <c r="C8">
+        <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="E8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>14</v>
       </c>
       <c r="B9" t="s">
         <v>15</v>
       </c>
-      <c r="C9" t="s">
-        <v>20</v>
+      <c r="C9">
+        <v>0</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>14</v>
       </c>
       <c r="B10" t="s">
         <v>16</v>
       </c>
-      <c r="C10" t="s">
-        <v>20</v>
+      <c r="C10">
+        <v>0</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>14</v>
       </c>
       <c r="B11" t="s">
         <v>17</v>
       </c>
-      <c r="C11" t="s">
-        <v>20</v>
+      <c r="C11">
+        <v>0</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="E11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>14</v>
       </c>
       <c r="B12" t="s">
         <v>18</v>
       </c>
-      <c r="C12" t="s">
-        <v>20</v>
+      <c r="C12">
+        <v>0</v>
       </c>
       <c r="D12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="E12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>14</v>
       </c>
       <c r="B13" t="s">
         <v>19</v>
       </c>
-      <c r="C13" t="s">
-        <v>20</v>
+      <c r="C13">
+        <v>0</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="E13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" t="s">
+        <v>21</v>
+      </c>
+      <c r="F20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
+        <v>46</v>
+      </c>
+      <c r="B25" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A28" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
+        <v>46</v>
+      </c>
+      <c r="B29" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+      <c r="D30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" t="s">
+        <v>54</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" t="s">
+        <v>21</v>
+      </c>
+      <c r="F31" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A32" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+      <c r="D32" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" t="s">
+        <v>21</v>
+      </c>
+      <c r="F32" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A33" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" t="s">
+        <v>56</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" t="s">
+        <v>21</v>
+      </c>
+      <c r="F33" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A34" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+      <c r="D34" t="s">
+        <v>20</v>
+      </c>
+      <c r="E34" t="s">
+        <v>21</v>
+      </c>
+      <c r="F34" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A35" t="s">
+        <v>52</v>
+      </c>
+      <c r="B35" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35" t="s">
+        <v>20</v>
+      </c>
+      <c r="E35" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A36" t="s">
+        <v>61</v>
+      </c>
+      <c r="B36" t="s">
+        <v>62</v>
+      </c>
+      <c r="C36">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A37" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" t="s">
+        <v>63</v>
+      </c>
+      <c r="C37">
+        <v>45</v>
+      </c>
+      <c r="D37" t="s">
+        <v>84</v>
+      </c>
+      <c r="E37" t="s">
+        <v>85</v>
+      </c>
+      <c r="F37" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A38" t="s">
+        <v>61</v>
+      </c>
+      <c r="B38" t="s">
+        <v>64</v>
+      </c>
+      <c r="C38">
+        <v>70</v>
+      </c>
+      <c r="D38" t="s">
+        <v>84</v>
+      </c>
+      <c r="E38" t="s">
+        <v>85</v>
+      </c>
+      <c r="F38" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A39" t="s">
+        <v>61</v>
+      </c>
+      <c r="B39" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39">
+        <v>90</v>
+      </c>
+      <c r="D39" t="s">
+        <v>84</v>
+      </c>
+      <c r="E39" t="s">
+        <v>85</v>
+      </c>
+      <c r="F39" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A40" t="s">
+        <v>61</v>
+      </c>
+      <c r="B40" t="s">
+        <v>66</v>
+      </c>
+      <c r="C40">
+        <v>50</v>
+      </c>
+      <c r="D40" t="s">
+        <v>84</v>
+      </c>
+      <c r="E40" t="s">
+        <v>85</v>
+      </c>
+      <c r="F40" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A41" t="s">
+        <v>61</v>
+      </c>
+      <c r="B41" t="s">
+        <v>67</v>
+      </c>
+      <c r="C41">
+        <v>65</v>
+      </c>
+      <c r="D41" t="s">
+        <v>84</v>
+      </c>
+      <c r="E41" t="s">
+        <v>85</v>
+      </c>
+      <c r="F41" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A42" t="s">
+        <v>61</v>
+      </c>
+      <c r="B42" t="s">
+        <v>68</v>
+      </c>
+      <c r="C42">
+        <v>50</v>
+      </c>
+      <c r="D42" t="s">
+        <v>84</v>
+      </c>
+      <c r="E42" t="s">
+        <v>85</v>
+      </c>
+      <c r="F42" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A43" t="s">
+        <v>61</v>
+      </c>
+      <c r="B43" t="s">
+        <v>69</v>
+      </c>
+      <c r="C43">
+        <v>65</v>
+      </c>
+      <c r="D43" t="s">
+        <v>84</v>
+      </c>
+      <c r="E43" t="s">
+        <v>85</v>
+      </c>
+      <c r="F43" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A44" t="s">
+        <v>61</v>
+      </c>
+      <c r="B44" t="s">
+        <v>70</v>
+      </c>
+      <c r="C44">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A45" t="s">
+        <v>61</v>
+      </c>
+      <c r="B45" t="s">
+        <v>71</v>
+      </c>
+      <c r="C45">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A46" t="s">
+        <v>61</v>
+      </c>
+      <c r="B46" t="s">
+        <v>72</v>
+      </c>
+      <c r="C46">
+        <v>85</v>
+      </c>
+      <c r="D46" t="s">
+        <v>90</v>
+      </c>
+      <c r="E46" t="s">
+        <v>85</v>
+      </c>
+      <c r="F46" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A47" t="s">
+        <v>61</v>
+      </c>
+      <c r="B47" t="s">
+        <v>73</v>
+      </c>
+      <c r="C47">
+        <v>85</v>
+      </c>
+      <c r="D47" t="s">
+        <v>90</v>
+      </c>
+      <c r="E47" t="s">
+        <v>85</v>
+      </c>
+      <c r="F47" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B48" t="s">
+        <v>74</v>
+      </c>
+      <c r="C48">
+        <v>85</v>
+      </c>
+      <c r="D48" t="s">
+        <v>90</v>
+      </c>
+      <c r="E48" t="s">
+        <v>85</v>
+      </c>
+      <c r="F48" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A49" t="s">
+        <v>61</v>
+      </c>
+      <c r="B49" t="s">
+        <v>75</v>
+      </c>
+      <c r="C49">
+        <v>85</v>
+      </c>
+      <c r="D49" t="s">
+        <v>90</v>
+      </c>
+      <c r="E49" t="s">
+        <v>85</v>
+      </c>
+      <c r="F49" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A50" t="s">
+        <v>61</v>
+      </c>
+      <c r="B50" t="s">
+        <v>76</v>
+      </c>
+      <c r="C50">
+        <v>88</v>
+      </c>
+      <c r="D50" t="s">
+        <v>90</v>
+      </c>
+      <c r="E50" t="s">
+        <v>85</v>
+      </c>
+      <c r="F50" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A51" t="s">
+        <v>61</v>
+      </c>
+      <c r="B51" t="s">
+        <v>77</v>
+      </c>
+      <c r="C51">
+        <v>88</v>
+      </c>
+      <c r="D51" t="s">
+        <v>90</v>
+      </c>
+      <c r="E51" t="s">
+        <v>85</v>
+      </c>
+      <c r="F51" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A52" t="s">
+        <v>61</v>
+      </c>
+      <c r="B52" t="s">
+        <v>78</v>
+      </c>
+      <c r="C52">
+        <v>88</v>
+      </c>
+      <c r="D52" t="s">
+        <v>90</v>
+      </c>
+      <c r="E52" t="s">
+        <v>85</v>
+      </c>
+      <c r="F52" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A53" t="s">
+        <v>61</v>
+      </c>
+      <c r="B53" t="s">
+        <v>79</v>
+      </c>
+      <c r="C53">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A54" t="s">
+        <v>61</v>
+      </c>
+      <c r="B54" t="s">
+        <v>80</v>
+      </c>
+      <c r="C54">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A55" t="s">
+        <v>61</v>
+      </c>
+      <c r="B55" t="s">
+        <v>81</v>
+      </c>
+      <c r="C55">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A56" t="s">
+        <v>61</v>
+      </c>
+      <c r="B56" t="s">
+        <v>82</v>
+      </c>
+      <c r="C56">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A57" t="s">
+        <v>61</v>
+      </c>
+      <c r="B57" t="s">
+        <v>83</v>
+      </c>
+      <c r="C57">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A58" t="s">
+        <v>92</v>
+      </c>
+      <c r="B58" t="s">
+        <v>93</v>
+      </c>
+      <c r="C58">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A59" t="s">
+        <v>92</v>
+      </c>
+      <c r="B59" t="s">
+        <v>94</v>
+      </c>
+      <c r="C59">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A60" t="s">
+        <v>92</v>
+      </c>
+      <c r="B60" t="s">
+        <v>95</v>
+      </c>
+      <c r="C60">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A61" t="s">
+        <v>92</v>
+      </c>
+      <c r="B61" t="s">
+        <v>96</v>
+      </c>
+      <c r="C61">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A62" t="s">
+        <v>92</v>
+      </c>
+      <c r="B62" t="s">
+        <v>97</v>
+      </c>
+      <c r="C62">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A63" t="s">
+        <v>98</v>
+      </c>
+      <c r="B63" t="s">
+        <v>99</v>
+      </c>
+      <c r="C63">
+        <v>0</v>
+      </c>
+      <c r="D63" t="s">
+        <v>20</v>
+      </c>
+      <c r="E63" t="s">
+        <v>21</v>
+      </c>
+      <c r="F63" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A64" t="s">
+        <v>98</v>
+      </c>
+      <c r="B64" t="s">
+        <v>100</v>
+      </c>
+      <c r="C64">
+        <v>0</v>
+      </c>
+      <c r="D64" t="s">
+        <v>20</v>
+      </c>
+      <c r="E64" t="s">
+        <v>21</v>
+      </c>
+      <c r="F64" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A65" t="s">
+        <v>98</v>
+      </c>
+      <c r="B65" t="s">
+        <v>101</v>
+      </c>
+      <c r="C65">
+        <v>0</v>
+      </c>
+      <c r="D65" t="s">
+        <v>20</v>
+      </c>
+      <c r="E65" t="s">
+        <v>21</v>
+      </c>
+      <c r="F65" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A66" t="s">
+        <v>98</v>
+      </c>
+      <c r="B66" t="s">
+        <v>102</v>
+      </c>
+      <c r="C66">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A67" t="s">
+        <v>98</v>
+      </c>
+      <c r="B67" t="s">
+        <v>103</v>
+      </c>
+      <c r="C67">
+        <v>0</v>
+      </c>
+      <c r="D67" t="s">
+        <v>20</v>
+      </c>
+      <c r="E67" t="s">
+        <v>21</v>
+      </c>
+      <c r="F67" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A68" t="s">
+        <v>98</v>
+      </c>
+      <c r="B68" t="s">
+        <v>104</v>
+      </c>
+      <c r="C68">
+        <v>0</v>
+      </c>
+      <c r="D68" t="s">
+        <v>20</v>
+      </c>
+      <c r="E68" t="s">
+        <v>21</v>
+      </c>
+      <c r="F68" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A69" t="s">
+        <v>98</v>
+      </c>
+      <c r="B69" t="s">
+        <v>105</v>
+      </c>
+      <c r="C69">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A70" t="s">
+        <v>111</v>
+      </c>
+      <c r="B70" t="s">
+        <v>112</v>
+      </c>
+      <c r="C70">
+        <v>0</v>
+      </c>
+      <c r="D70" t="s">
+        <v>20</v>
+      </c>
+      <c r="E70" t="s">
+        <v>21</v>
+      </c>
+      <c r="F70" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A71" t="s">
+        <v>111</v>
+      </c>
+      <c r="B71" t="s">
+        <v>113</v>
+      </c>
+      <c r="C71">
+        <v>0</v>
+      </c>
+      <c r="D71" t="s">
+        <v>20</v>
+      </c>
+      <c r="E71" t="s">
+        <v>21</v>
+      </c>
+      <c r="F71" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A72" t="s">
+        <v>111</v>
+      </c>
+      <c r="B72" t="s">
+        <v>114</v>
+      </c>
+      <c r="C72">
+        <v>0</v>
+      </c>
+      <c r="D72" t="s">
+        <v>20</v>
+      </c>
+      <c r="E72" t="s">
+        <v>21</v>
+      </c>
+      <c r="F72" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A73" t="s">
+        <v>111</v>
+      </c>
+      <c r="B73" t="s">
+        <v>115</v>
+      </c>
+      <c r="C73">
+        <v>0</v>
+      </c>
+      <c r="D73" t="s">
+        <v>20</v>
+      </c>
+      <c r="E73" t="s">
+        <v>21</v>
+      </c>
+      <c r="F73" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A74" t="s">
+        <v>111</v>
+      </c>
+      <c r="B74" t="s">
+        <v>116</v>
+      </c>
+      <c r="C74">
+        <v>0</v>
+      </c>
+      <c r="D74" t="s">
+        <v>20</v>
+      </c>
+      <c r="E74" t="s">
+        <v>21</v>
+      </c>
+      <c r="F74" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A75" t="s">
+        <v>111</v>
+      </c>
+      <c r="B75" t="s">
+        <v>117</v>
+      </c>
+      <c r="C75">
+        <v>0</v>
+      </c>
+      <c r="D75" t="s">
+        <v>20</v>
+      </c>
+      <c r="E75" t="s">
+        <v>21</v>
+      </c>
+      <c r="F75" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A76" t="s">
+        <v>111</v>
+      </c>
+      <c r="B76" t="s">
+        <v>118</v>
+      </c>
+      <c r="C76">
+        <v>0</v>
+      </c>
+      <c r="D76" t="s">
+        <v>20</v>
+      </c>
+      <c r="E76" t="s">
+        <v>21</v>
+      </c>
+      <c r="F76" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A77" t="s">
+        <v>111</v>
+      </c>
+      <c r="B77" t="s">
+        <v>119</v>
+      </c>
+      <c r="C77">
+        <v>0</v>
+      </c>
+      <c r="D77" t="s">
+        <v>20</v>
+      </c>
+      <c r="E77" t="s">
+        <v>21</v>
+      </c>
+      <c r="F77" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A78" t="s">
+        <v>111</v>
+      </c>
+      <c r="B78" t="s">
+        <v>120</v>
+      </c>
+      <c r="C78">
+        <v>0</v>
+      </c>
+      <c r="D78" t="s">
+        <v>20</v>
+      </c>
+      <c r="E78" t="s">
+        <v>21</v>
+      </c>
+      <c r="F78" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A79" t="s">
+        <v>111</v>
+      </c>
+      <c r="B79" t="s">
+        <v>121</v>
+      </c>
+      <c r="C79">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A80" t="s">
+        <v>111</v>
+      </c>
+      <c r="B80" t="s">
+        <v>122</v>
+      </c>
+      <c r="C80">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>